<commit_message>
Expand Reader vocabulary template and remove X dropdowns
</commit_message>
<xml_diff>
--- a/PeninaPlus-Reader/Vocabulary_By_Category.xlsx
+++ b/PeninaPlus-Reader/Vocabulary_By_Category.xlsx
@@ -2,10 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbs" sheetId="1" r:id="R17632715b5f147af"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nouns" sheetId="2" r:id="R0dcc5ccf54ef47ee"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjectives" sheetId="3" r:id="Rb1a2e48d035f4479"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R53aa0339a5e44e11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbs" sheetId="1" r:id="R23291a9596294f64"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nouns" sheetId="2" r:id="Rd42b20cfdab54524"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjectives" sheetId="3" r:id="R90b52fff8f6b489f"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Re3f6db3c23b642bf"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prepositions" sheetId="5" r:id="Rd06b240a5c6a4df5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adverbs" sheetId="6" r:id="Rfbb4b3a09ef94d71"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conjunctions" sheetId="7" r:id="R79fa3d69eeb04f88"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Words" sheetId="8" r:id="R089a6ce5a5ff4330"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phrases &amp; Expressions" sheetId="9" r:id="R33959c7c6c084e94"/>
   </sheets>
 </workbook>
 </file>
@@ -556,11 +561,6 @@
       <c r="H21" s="5"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="C2:H1000">
-      <formula1>"X"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -781,7 +781,7 @@
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="7" t="str">
-        <v>Keep the sheet names Verbs, Nouns, and Adjectives. Unused sheets may be left empty or removed.</v>
+        <v>Keep the sheet names unchanged. Unused sheets may be left empty or removed.</v>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
@@ -813,6 +813,416 @@
       <c r="A8" s="7" t="str">
         <v>In the Reader, select the noun categories you want to include. Duplicate words are combined.</v>
       </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="str">
+        <v>Prepositions: enter one mastered Hebrew preposition per cell below the heading.</v>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="7" t="str">
+        <v>Adverbs: enter one mastered Hebrew adverb per cell below the heading.</v>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="7" t="str">
+        <v>Conjunctions: enter one mastered Hebrew conjunction per cell below the heading.</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="7" t="str">
+        <v>Question Words: enter one mastered Hebrew question word per cell below the heading.</v>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="7" t="str">
+        <v>Phrases &amp; Expressions: enter one complete Hebrew phrase per cell, with spaces between its words.</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>מילות יחס</v>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="5"/>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="5"/>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="5"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="5"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="5"/>
+    </row>
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="5"/>
+    </row>
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="5"/>
+    </row>
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="5"/>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="5"/>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="5"/>
+    </row>
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" s="5"/>
+    </row>
+    <row r="14" ht="25" customHeight="1">
+      <c r="A14" s="5"/>
+    </row>
+    <row r="15" ht="25" customHeight="1">
+      <c r="A15" s="5"/>
+    </row>
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="5"/>
+    </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="5"/>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="5"/>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="5"/>
+    </row>
+    <row r="21" ht="25" customHeight="1">
+      <c r="A21" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>תוארי פועל</v>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="5"/>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="5"/>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="5"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="5"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="5"/>
+    </row>
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="5"/>
+    </row>
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="5"/>
+    </row>
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="5"/>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="5"/>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="5"/>
+    </row>
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" s="5"/>
+    </row>
+    <row r="14" ht="25" customHeight="1">
+      <c r="A14" s="5"/>
+    </row>
+    <row r="15" ht="25" customHeight="1">
+      <c r="A15" s="5"/>
+    </row>
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="5"/>
+    </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="5"/>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="5"/>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="5"/>
+    </row>
+    <row r="21" ht="25" customHeight="1">
+      <c r="A21" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>מילות קישור</v>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="5"/>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="5"/>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="5"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="5"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="5"/>
+    </row>
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="5"/>
+    </row>
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="5"/>
+    </row>
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="5"/>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="5"/>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="5"/>
+    </row>
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" s="5"/>
+    </row>
+    <row r="14" ht="25" customHeight="1">
+      <c r="A14" s="5"/>
+    </row>
+    <row r="15" ht="25" customHeight="1">
+      <c r="A15" s="5"/>
+    </row>
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="5"/>
+    </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="5"/>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="5"/>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="5"/>
+    </row>
+    <row r="21" ht="25" customHeight="1">
+      <c r="A21" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>מילות שאלה</v>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="5"/>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="5"/>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="5"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="5"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="5"/>
+    </row>
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="5"/>
+    </row>
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="5"/>
+    </row>
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="5"/>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="5"/>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="5"/>
+    </row>
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" s="5"/>
+    </row>
+    <row r="14" ht="25" customHeight="1">
+      <c r="A14" s="5"/>
+    </row>
+    <row r="15" ht="25" customHeight="1">
+      <c r="A15" s="5"/>
+    </row>
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="5"/>
+    </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="5"/>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="5"/>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="5"/>
+    </row>
+    <row r="21" ht="25" customHeight="1">
+      <c r="A21" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>ביטויים וצירופים</v>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="5"/>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="5"/>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="5"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="5"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="5"/>
+    </row>
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="5"/>
+    </row>
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="5"/>
+    </row>
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="5"/>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="5"/>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="5"/>
+    </row>
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" s="5"/>
+    </row>
+    <row r="14" ht="25" customHeight="1">
+      <c r="A14" s="5"/>
+    </row>
+    <row r="15" ht="25" customHeight="1">
+      <c r="A15" s="5"/>
+    </row>
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="5"/>
+    </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="5"/>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="5"/>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="5"/>
+    </row>
+    <row r="21" ht="25" customHeight="1">
+      <c r="A21" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Refine Reader workbook, defaults, question controls and exports
</commit_message>
<xml_diff>
--- a/PeninaPlus-Reader/Vocabulary_By_Category.xlsx
+++ b/PeninaPlus-Reader/Vocabulary_By_Category.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbs" sheetId="1" r:id="R23291a9596294f64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nouns" sheetId="2" r:id="Rd42b20cfdab54524"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjectives" sheetId="3" r:id="R90b52fff8f6b489f"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Re3f6db3c23b642bf"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prepositions" sheetId="5" r:id="Rd06b240a5c6a4df5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adverbs" sheetId="6" r:id="Rfbb4b3a09ef94d71"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conjunctions" sheetId="7" r:id="R79fa3d69eeb04f88"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Words" sheetId="8" r:id="R089a6ce5a5ff4330"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phrases &amp; Expressions" sheetId="9" r:id="R33959c7c6c084e94"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbs" sheetId="1" r:id="R10a98d563f0345a6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nouns" sheetId="2" r:id="Rb1241042ad8744ff"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjectives" sheetId="3" r:id="R21fe178b0a664c1d"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prepositions" sheetId="5" r:id="R972bc8955a004168"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adverbs" sheetId="6" r:id="Rb2bb2f3e4bb04d64"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conjunctions" sheetId="7" r:id="Rc33cbca83b434e89"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Words" sheetId="8" r:id="R2ef9d52211074f10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phrases &amp; Expressions" sheetId="9" r:id="Rbb0eeaf6e3e1400a"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R295af02a88cc4617"/>
   </sheets>
 </workbook>
 </file>
@@ -60,7 +60,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -68,11 +68,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9DEE3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9DEE3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9DEE3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9DEE3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -95,6 +110,24 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -309,256 +342,256 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="11" t="str">
         <v>שורשים</v>
       </c>
-      <c r="B1" s="4" t="str">
+      <c r="B1" s="11" t="str">
         <v>בניין</v>
       </c>
-      <c r="C1" s="4" t="str">
+      <c r="C1" s="11" t="str">
         <v>עבר</v>
       </c>
-      <c r="D1" s="4" t="str">
+      <c r="D1" s="11" t="str">
         <v>הווה</v>
       </c>
-      <c r="E1" s="4" t="str">
+      <c r="E1" s="11" t="str">
         <v>עתיד</v>
       </c>
-      <c r="F1" s="4" t="str">
+      <c r="F1" s="11" t="str">
         <v>שם הפועל</v>
       </c>
-      <c r="G1" s="4" t="str">
+      <c r="G1" s="11" t="str">
         <v>שם פעולה</v>
       </c>
-      <c r="H1" s="4" t="str">
+      <c r="H1" s="11" t="str">
         <v>ציווי</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5" t="str">
+      <c r="A2" s="10"/>
+      <c r="B2" s="10" t="str">
         <v>פעל שלם</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5" t="str">
+      <c r="A3" s="10"/>
+      <c r="B3" s="10" t="str">
         <v>פעל ל-ה</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5" t="str">
+      <c r="A4" s="10"/>
+      <c r="B4" s="10" t="str">
         <v>פעל ע"ו</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
     </row>
     <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5" t="str">
+      <c r="A5" s="10"/>
+      <c r="B5" s="10" t="str">
         <v>פעל חפ"נ</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
     </row>
     <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5" t="str">
+      <c r="A6" s="10"/>
+      <c r="B6" s="10" t="str">
         <v>פעל פ"י</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5" t="str">
+      <c r="A7" s="10"/>
+      <c r="B7" s="10" t="str">
         <v>פיעל שלם</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
     </row>
     <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5" t="str">
+      <c r="A8" s="10"/>
+      <c r="B8" s="10" t="str">
         <v>פיעל ל-ה</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
     </row>
     <row r="9" ht="25" customHeight="1">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5" t="str">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10" t="str">
         <v>הפעיל שלם</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
     </row>
     <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5" t="str">
+      <c r="A10" s="10"/>
+      <c r="B10" s="10" t="str">
         <v>הפעיל ל-ה</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5" t="str">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10" t="str">
         <v>הפעיל ע"ו</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
     </row>
     <row r="12" ht="25" customHeight="1">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5" t="str">
+      <c r="A12" s="10"/>
+      <c r="B12" s="10" t="str">
         <v>הפעיל פ"י</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
     </row>
     <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5" t="str">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10" t="str">
         <v>התפעל שלם</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
     </row>
     <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5" t="str">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10" t="str">
         <v>נפעל שלם</v>
       </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
     </row>
     <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
     </row>
     <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
     </row>
     <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
     </row>
     <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
     </row>
     <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
     </row>
     <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
     </row>
     <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -575,115 +608,115 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="11" t="str">
         <v>Clothing</v>
       </c>
-      <c r="B1" s="4" t="str">
+      <c r="B1" s="11" t="str">
         <v>Body parts</v>
       </c>
-      <c r="C1" s="4" t="str">
+      <c r="C1" s="11" t="str">
         <v>Animals</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
+      <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
     </row>
     <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
     </row>
     <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
     </row>
     <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
     </row>
     <row r="9" ht="25" customHeight="1">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
     </row>
     <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
     </row>
     <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
     </row>
     <row r="12" ht="25" customHeight="1">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
     </row>
     <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
     </row>
     <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
     </row>
     <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
     </row>
     <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
     </row>
     <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
     </row>
     <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
     </row>
     <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
     </row>
     <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
     </row>
     <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -698,69 +731,69 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="11" t="str">
         <v>שם תואר</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="5"/>
+      <c r="A2" s="10"/>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="5"/>
+      <c r="A3" s="10"/>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="5"/>
+      <c r="A4" s="10"/>
     </row>
     <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="5"/>
+      <c r="A5" s="10"/>
     </row>
     <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="5"/>
+      <c r="A6" s="10"/>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="5"/>
+      <c r="A7" s="10"/>
     </row>
     <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="5"/>
+      <c r="A8" s="10"/>
     </row>
     <row r="9" ht="25" customHeight="1">
-      <c r="A9" s="5"/>
+      <c r="A9" s="10"/>
     </row>
     <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="5"/>
+      <c r="A10" s="10"/>
     </row>
     <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="5"/>
+      <c r="A11" s="10"/>
     </row>
     <row r="12" ht="25" customHeight="1">
-      <c r="A12" s="5"/>
+      <c r="A12" s="10"/>
     </row>
     <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="5"/>
+      <c r="A13" s="10"/>
     </row>
     <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="5"/>
+      <c r="A14" s="10"/>
     </row>
     <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="5"/>
+      <c r="A15" s="10"/>
     </row>
     <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="5"/>
+      <c r="A16" s="10"/>
     </row>
     <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="5"/>
+      <c r="A17" s="10"/>
     </row>
     <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="5"/>
+      <c r="A18" s="10"/>
     </row>
     <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="5"/>
+      <c r="A19" s="10"/>
     </row>
     <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="5"/>
+      <c r="A20" s="10"/>
     </row>
     <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="5"/>
+      <c r="A21" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -775,67 +808,67 @@
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="8" t="str">
+      <c r="A1" s="14" t="str">
         <v>Vocabulary workbook</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="7" t="str">
+      <c r="A2" s="13" t="str">
         <v>Keep the sheet names unchanged. Unused sheets may be left empty or removed.</v>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="7" t="str">
+      <c r="A3" s="13" t="str">
         <v>Verbs: enter roots in column A. In columns C–H, mark X beside each mastered verb pattern in column B.</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="7" t="str">
+      <c r="A4" s="13" t="str">
         <v>Nouns: rename or add category headings in row 1. Enter one Hebrew noun per cell below each heading.</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="7" t="str">
+      <c r="A5" s="13" t="str">
         <v>Use singular nouns. Categories can have different lengths. Blank cells are ignored.</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="7" t="str">
+      <c r="A6" s="13" t="str">
         <v>Adjectives: enter masculine singular Hebrew adjectives below the heading.</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="7" t="str">
-        <v>Upload this workbook, or select separate workbooks together. Each new upload replaces the previous selection.</v>
+      <c r="A7" s="13" t="str">
+        <v>Upload this single workbook with all your vocabulary sheets. Each new upload replaces the previous selection.</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="7" t="str">
+      <c r="A8" s="13" t="str">
         <v>In the Reader, select the noun categories you want to include. Duplicate words are combined.</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="str">
+      <c r="A9" s="13" t="str">
         <v>Prepositions: enter one mastered Hebrew preposition per cell below the heading.</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="7" t="str">
+      <c r="A10" s="13" t="str">
         <v>Adverbs: enter one mastered Hebrew adverb per cell below the heading.</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="7" t="str">
+      <c r="A11" s="13" t="str">
         <v>Conjunctions: enter one mastered Hebrew conjunction per cell below the heading.</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="7" t="str">
+      <c r="A12" s="13" t="str">
         <v>Question Words: enter one mastered Hebrew question word per cell below the heading.</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="7" t="str">
+      <c r="A13" s="13" t="str">
         <v>Phrases &amp; Expressions: enter one complete Hebrew phrase per cell, with spaces between its words.</v>
       </c>
     </row>
@@ -852,69 +885,69 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="11" t="str">
         <v>מילות יחס</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="5"/>
+      <c r="A2" s="10"/>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="5"/>
+      <c r="A3" s="10"/>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="5"/>
+      <c r="A4" s="10"/>
     </row>
     <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="5"/>
+      <c r="A5" s="10"/>
     </row>
     <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="5"/>
+      <c r="A6" s="10"/>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="5"/>
+      <c r="A7" s="10"/>
     </row>
     <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="5"/>
+      <c r="A8" s="10"/>
     </row>
     <row r="9" ht="25" customHeight="1">
-      <c r="A9" s="5"/>
+      <c r="A9" s="10"/>
     </row>
     <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="5"/>
+      <c r="A10" s="10"/>
     </row>
     <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="5"/>
+      <c r="A11" s="10"/>
     </row>
     <row r="12" ht="25" customHeight="1">
-      <c r="A12" s="5"/>
+      <c r="A12" s="10"/>
     </row>
     <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="5"/>
+      <c r="A13" s="10"/>
     </row>
     <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="5"/>
+      <c r="A14" s="10"/>
     </row>
     <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="5"/>
+      <c r="A15" s="10"/>
     </row>
     <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="5"/>
+      <c r="A16" s="10"/>
     </row>
     <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="5"/>
+      <c r="A17" s="10"/>
     </row>
     <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="5"/>
+      <c r="A18" s="10"/>
     </row>
     <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="5"/>
+      <c r="A19" s="10"/>
     </row>
     <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="5"/>
+      <c r="A20" s="10"/>
     </row>
     <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="5"/>
+      <c r="A21" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -929,69 +962,69 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="11" t="str">
         <v>תוארי פועל</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="5"/>
+      <c r="A2" s="10"/>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="5"/>
+      <c r="A3" s="10"/>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="5"/>
+      <c r="A4" s="10"/>
     </row>
     <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="5"/>
+      <c r="A5" s="10"/>
     </row>
     <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="5"/>
+      <c r="A6" s="10"/>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="5"/>
+      <c r="A7" s="10"/>
     </row>
     <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="5"/>
+      <c r="A8" s="10"/>
     </row>
     <row r="9" ht="25" customHeight="1">
-      <c r="A9" s="5"/>
+      <c r="A9" s="10"/>
     </row>
     <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="5"/>
+      <c r="A10" s="10"/>
     </row>
     <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="5"/>
+      <c r="A11" s="10"/>
     </row>
     <row r="12" ht="25" customHeight="1">
-      <c r="A12" s="5"/>
+      <c r="A12" s="10"/>
     </row>
     <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="5"/>
+      <c r="A13" s="10"/>
     </row>
     <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="5"/>
+      <c r="A14" s="10"/>
     </row>
     <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="5"/>
+      <c r="A15" s="10"/>
     </row>
     <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="5"/>
+      <c r="A16" s="10"/>
     </row>
     <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="5"/>
+      <c r="A17" s="10"/>
     </row>
     <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="5"/>
+      <c r="A18" s="10"/>
     </row>
     <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="5"/>
+      <c r="A19" s="10"/>
     </row>
     <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="5"/>
+      <c r="A20" s="10"/>
     </row>
     <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="5"/>
+      <c r="A21" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1006,69 +1039,69 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="11" t="str">
         <v>מילות קישור</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="5"/>
+      <c r="A2" s="10"/>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="5"/>
+      <c r="A3" s="10"/>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="5"/>
+      <c r="A4" s="10"/>
     </row>
     <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="5"/>
+      <c r="A5" s="10"/>
     </row>
     <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="5"/>
+      <c r="A6" s="10"/>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="5"/>
+      <c r="A7" s="10"/>
     </row>
     <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="5"/>
+      <c r="A8" s="10"/>
     </row>
     <row r="9" ht="25" customHeight="1">
-      <c r="A9" s="5"/>
+      <c r="A9" s="10"/>
     </row>
     <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="5"/>
+      <c r="A10" s="10"/>
     </row>
     <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="5"/>
+      <c r="A11" s="10"/>
     </row>
     <row r="12" ht="25" customHeight="1">
-      <c r="A12" s="5"/>
+      <c r="A12" s="10"/>
     </row>
     <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="5"/>
+      <c r="A13" s="10"/>
     </row>
     <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="5"/>
+      <c r="A14" s="10"/>
     </row>
     <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="5"/>
+      <c r="A15" s="10"/>
     </row>
     <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="5"/>
+      <c r="A16" s="10"/>
     </row>
     <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="5"/>
+      <c r="A17" s="10"/>
     </row>
     <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="5"/>
+      <c r="A18" s="10"/>
     </row>
     <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="5"/>
+      <c r="A19" s="10"/>
     </row>
     <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="5"/>
+      <c r="A20" s="10"/>
     </row>
     <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="5"/>
+      <c r="A21" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1083,69 +1116,69 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="11" t="str">
         <v>מילות שאלה</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="5"/>
+      <c r="A2" s="10"/>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="5"/>
+      <c r="A3" s="10"/>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="5"/>
+      <c r="A4" s="10"/>
     </row>
     <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="5"/>
+      <c r="A5" s="10"/>
     </row>
     <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="5"/>
+      <c r="A6" s="10"/>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="5"/>
+      <c r="A7" s="10"/>
     </row>
     <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="5"/>
+      <c r="A8" s="10"/>
     </row>
     <row r="9" ht="25" customHeight="1">
-      <c r="A9" s="5"/>
+      <c r="A9" s="10"/>
     </row>
     <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="5"/>
+      <c r="A10" s="10"/>
     </row>
     <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="5"/>
+      <c r="A11" s="10"/>
     </row>
     <row r="12" ht="25" customHeight="1">
-      <c r="A12" s="5"/>
+      <c r="A12" s="10"/>
     </row>
     <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="5"/>
+      <c r="A13" s="10"/>
     </row>
     <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="5"/>
+      <c r="A14" s="10"/>
     </row>
     <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="5"/>
+      <c r="A15" s="10"/>
     </row>
     <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="5"/>
+      <c r="A16" s="10"/>
     </row>
     <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="5"/>
+      <c r="A17" s="10"/>
     </row>
     <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="5"/>
+      <c r="A18" s="10"/>
     </row>
     <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="5"/>
+      <c r="A19" s="10"/>
     </row>
     <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="5"/>
+      <c r="A20" s="10"/>
     </row>
     <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="5"/>
+      <c r="A21" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1160,69 +1193,69 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="11" t="str">
         <v>ביטויים וצירופים</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="5"/>
+      <c r="A2" s="10"/>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="5"/>
+      <c r="A3" s="10"/>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="5"/>
+      <c r="A4" s="10"/>
     </row>
     <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="5"/>
+      <c r="A5" s="10"/>
     </row>
     <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="5"/>
+      <c r="A6" s="10"/>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="5"/>
+      <c r="A7" s="10"/>
     </row>
     <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="5"/>
+      <c r="A8" s="10"/>
     </row>
     <row r="9" ht="25" customHeight="1">
-      <c r="A9" s="5"/>
+      <c r="A9" s="10"/>
     </row>
     <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="5"/>
+      <c r="A10" s="10"/>
     </row>
     <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="5"/>
+      <c r="A11" s="10"/>
     </row>
     <row r="12" ht="25" customHeight="1">
-      <c r="A12" s="5"/>
+      <c r="A12" s="10"/>
     </row>
     <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="5"/>
+      <c r="A13" s="10"/>
     </row>
     <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="5"/>
+      <c r="A14" s="10"/>
     </row>
     <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="5"/>
+      <c r="A15" s="10"/>
     </row>
     <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="5"/>
+      <c r="A16" s="10"/>
     </row>
     <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="5"/>
+      <c r="A17" s="10"/>
     </row>
     <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="5"/>
+      <c r="A18" s="10"/>
     </row>
     <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="5"/>
+      <c r="A19" s="10"/>
     </row>
     <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="5"/>
+      <c r="A20" s="10"/>
     </row>
     <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="5"/>
+      <c r="A21" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add adjective category columns and independent category selection
</commit_message>
<xml_diff>
--- a/PeninaPlus-Reader/Vocabulary_By_Category.xlsx
+++ b/PeninaPlus-Reader/Vocabulary_By_Category.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbs" sheetId="1" r:id="R10a98d563f0345a6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nouns" sheetId="2" r:id="Rb1241042ad8744ff"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjectives" sheetId="3" r:id="R21fe178b0a664c1d"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prepositions" sheetId="5" r:id="R972bc8955a004168"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adverbs" sheetId="6" r:id="Rb2bb2f3e4bb04d64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conjunctions" sheetId="7" r:id="Rc33cbca83b434e89"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Words" sheetId="8" r:id="R2ef9d52211074f10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phrases &amp; Expressions" sheetId="9" r:id="Rbb0eeaf6e3e1400a"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R295af02a88cc4617"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbs" sheetId="1" r:id="R8aa4fe2dcb064d1e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nouns" sheetId="2" r:id="R9115db9ec4b74e12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjectives" sheetId="3" r:id="Reecfb849b2a04100"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prepositions" sheetId="5" r:id="R3916e95b96d74b19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adverbs" sheetId="6" r:id="Refcfb413dbf84520"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conjunctions" sheetId="7" r:id="R8adc9fceac964b45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Words" sheetId="8" r:id="R39b6d5419fb54fe6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phrases &amp; Expressions" sheetId="9" r:id="R8b423743b63d4c5b"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Ra4397e34da9343ce"/>
   </sheets>
 </workbook>
 </file>
@@ -727,73 +727,169 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="22" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="11" t="str">
-        <v>שם תואר</v>
+        <v>Size</v>
+      </c>
+      <c r="B1" s="11" t="str">
+        <v>Color</v>
+      </c>
+      <c r="C1" s="11" t="str">
+        <v>Shape</v>
+      </c>
+      <c r="D1" s="11" t="str">
+        <v>Feelings</v>
+      </c>
+      <c r="E1" s="11" t="str">
+        <v>Qualities</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
     </row>
     <row r="7" ht="25" customHeight="1">
       <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
     </row>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
     </row>
     <row r="11" ht="25" customHeight="1">
       <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
     </row>
     <row r="12" ht="25" customHeight="1">
       <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
     </row>
     <row r="13" ht="25" customHeight="1">
       <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
     </row>
     <row r="14" ht="25" customHeight="1">
       <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
     </row>
     <row r="15" ht="25" customHeight="1">
       <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
     </row>
     <row r="16" ht="25" customHeight="1">
       <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
     </row>
     <row r="17" ht="25" customHeight="1">
       <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
     </row>
     <row r="18" ht="25" customHeight="1">
       <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
     </row>
     <row r="19" ht="25" customHeight="1">
       <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -804,73 +900,73 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="115" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="19" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="14" t="str">
-        <v>Vocabulary workbook</v>
-      </c>
-    </row>
-    <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="13" t="str">
-        <v>Keep the sheet names unchanged. Unused sheets may be left empty or removed.</v>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="13" t="str">
-        <v>Verbs: enter roots in column A. In columns C–H, mark X beside each mastered verb pattern in column B.</v>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="13" t="str">
-        <v>Nouns: rename or add category headings in row 1. Enter one Hebrew noun per cell below each heading.</v>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="13" t="str">
-        <v>Use singular nouns. Categories can have different lengths. Blank cells are ignored.</v>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="13" t="str">
-        <v>Adjectives: enter masculine singular Hebrew adjectives below the heading.</v>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="13" t="str">
-        <v>Upload this single workbook with all your vocabulary sheets. Each new upload replaces the previous selection.</v>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="13" t="str">
-        <v>In the Reader, select the noun categories you want to include. Duplicate words are combined.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="str">
-        <v>Prepositions: enter one mastered Hebrew preposition per cell below the heading.</v>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="13" t="str">
-        <v>Adverbs: enter one mastered Hebrew adverb per cell below the heading.</v>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="13" t="str">
-        <v>Conjunctions: enter one mastered Hebrew conjunction per cell below the heading.</v>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="13" t="str">
-        <v>Question Words: enter one mastered Hebrew question word per cell below the heading.</v>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="13" t="str">
-        <v>Phrases &amp; Expressions: enter one complete Hebrew phrase per cell, with spaces between its words.</v>
-      </c>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="11" t="str">
+        <v>מילות יחס</v>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="10"/>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="10"/>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="10"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="10"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="10"/>
+    </row>
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="10"/>
+    </row>
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="10"/>
+    </row>
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="10"/>
+    </row>
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="10"/>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="10"/>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="10"/>
+    </row>
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" s="10"/>
+    </row>
+    <row r="14" ht="25" customHeight="1">
+      <c r="A14" s="10"/>
+    </row>
+    <row r="15" ht="25" customHeight="1">
+      <c r="A15" s="10"/>
+    </row>
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="10"/>
+    </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="10"/>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="10"/>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="10"/>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="10"/>
+    </row>
+    <row r="21" ht="25" customHeight="1">
+      <c r="A21" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -881,12 +977,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="24" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="11" t="str">
-        <v>מילות יחס</v>
+        <v>תוארי פועל</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
@@ -963,7 +1059,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="11" t="str">
-        <v>תוארי פועל</v>
+        <v>מילות קישור</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
@@ -1040,7 +1136,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="11" t="str">
-        <v>מילות קישור</v>
+        <v>מילות שאלה</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
@@ -1112,12 +1208,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="42" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="11" t="str">
-        <v>מילות שאלה</v>
+        <v>ביטויים וצירופים</v>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
@@ -1189,73 +1285,73 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="115" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="11" t="str">
-        <v>ביטויים וצירופים</v>
-      </c>
-    </row>
-    <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="10"/>
-    </row>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="10"/>
-    </row>
-    <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="10"/>
-    </row>
-    <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="10"/>
-    </row>
-    <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="10"/>
-    </row>
-    <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="10"/>
-    </row>
-    <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="10"/>
-    </row>
-    <row r="9" ht="25" customHeight="1">
-      <c r="A9" s="10"/>
-    </row>
-    <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="10"/>
-    </row>
-    <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="10"/>
-    </row>
-    <row r="12" ht="25" customHeight="1">
-      <c r="A12" s="10"/>
-    </row>
-    <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="10"/>
-    </row>
-    <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="10"/>
-    </row>
-    <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="10"/>
-    </row>
-    <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="10"/>
-    </row>
-    <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="10"/>
-    </row>
-    <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="10"/>
-    </row>
-    <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="10"/>
-    </row>
-    <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="10"/>
-    </row>
-    <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="10"/>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="14" t="str">
+        <v>Vocabulary workbook</v>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="13" t="str">
+        <v>Keep the sheet names unchanged. Unused sheets may be left empty or removed.</v>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="13" t="str">
+        <v>Verbs: enter roots in column A. In columns C–H, mark X beside each mastered verb pattern in column B.</v>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="13" t="str">
+        <v>Nouns: rename or add category headings in row 1. Enter one Hebrew noun per cell below each heading.</v>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="13" t="str">
+        <v>Use singular nouns. Categories can have different lengths. Blank cells are ignored.</v>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="13" t="str">
+        <v>Adjectives: rename or add category columns in row 1. Enter one masculine singular Hebrew adjective per cell.</v>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="13" t="str">
+        <v>Upload this single workbook with all your vocabulary sheets. Each new upload replaces the previous selection.</v>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="13" t="str">
+        <v>In the Reader, select the noun and adjective categories to include. Duplicate words are combined.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="str">
+        <v>Prepositions: enter one mastered Hebrew preposition per cell below the heading.</v>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="13" t="str">
+        <v>Adverbs: enter one mastered Hebrew adverb per cell below the heading.</v>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="13" t="str">
+        <v>Conjunctions: enter one mastered Hebrew conjunction per cell below the heading.</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="13" t="str">
+        <v>Question Words: enter one mastered Hebrew question word per cell below the heading.</v>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="13" t="str">
+        <v>Phrases &amp; Expressions: enter one complete Hebrew phrase per cell, with spaces between its words.</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>